<commit_message>
fix: typos in team stats scripts
</commit_message>
<xml_diff>
--- a/app/team_stats_2024.xlsx
+++ b/app/team_stats_2024.xlsx
@@ -539,7 +539,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C2" s="1" t="n">
@@ -596,7 +596,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C3" s="1" t="n">
@@ -653,7 +653,7 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C4" s="1" t="n">
@@ -710,7 +710,7 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C5" s="1" t="n">
@@ -767,7 +767,7 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C6" s="1" t="n">
@@ -866,7 +866,7 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C9" s="1" t="n">
@@ -923,7 +923,7 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C10" s="1" t="n">
@@ -980,7 +980,7 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C11" s="1" t="n">
@@ -1079,7 +1079,7 @@
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C14" s="1" t="n">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C15" s="1" t="n">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C16" s="1" t="n">
@@ -1250,7 +1250,7 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C17" s="1" t="n">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C18" s="1" t="n">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C19" s="1" t="n">
@@ -1421,7 +1421,7 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C20" s="1" t="n">
@@ -1520,7 +1520,7 @@
       </c>
       <c r="B23" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C23" s="1" t="n">
@@ -1577,7 +1577,7 @@
       </c>
       <c r="B24" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C24" s="1" t="n">
@@ -1634,7 +1634,7 @@
       </c>
       <c r="B25" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C25" s="1" t="n">
@@ -1691,7 +1691,7 @@
       </c>
       <c r="B26" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C26" s="1" t="n">
@@ -1748,7 +1748,7 @@
       </c>
       <c r="B27" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C27" s="1" t="n">
@@ -1805,7 +1805,7 @@
       </c>
       <c r="B28" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C28" s="1" t="n">
@@ -1904,7 +1904,7 @@
       </c>
       <c r="B31" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C31" s="1" t="n">
@@ -1961,7 +1961,7 @@
       </c>
       <c r="B32" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C32" s="1" t="n">
@@ -2018,7 +2018,7 @@
       </c>
       <c r="B33" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C33" s="1" t="n">
@@ -2075,7 +2075,7 @@
       </c>
       <c r="B34" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C34" s="1" t="n">
@@ -2132,7 +2132,7 @@
       </c>
       <c r="B35" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C35" s="1" t="n">
@@ -2189,7 +2189,7 @@
       </c>
       <c r="B36" s="1" t="inlineStr">
         <is>
-          <t>2025/2026</t>
+          <t>2024/2025</t>
         </is>
       </c>
       <c r="C36" s="1" t="n">

</xml_diff>